<commit_message>
final included studies extraction
</commit_message>
<xml_diff>
--- a/results/full_text/full_text_eligibility_agent.xlsx
+++ b/results/full_text/full_text_eligibility_agent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason\Projects\srma-agent-toolkit\results\full_text\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B53392-0DD7-466A-AE26-92EC4791FB61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AF42C6-4F35-4205-B2BA-1C9B589D1DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="28920" windowHeight="15600" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -22,11 +22,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Author_Final_Review!$A$3:$W$33</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="479">
   <si>
     <t>Efficacy and safety of preoperative or perioperative SGLT2 inhibitors in adult cardiac surgery: a systematic review and meta-analysis — Full-Text Eligibility</t>
   </si>
@@ -1348,11 +1353,544 @@
     <t>Full text not available</t>
   </si>
   <si>
-    <t>Empagliflozin limits AKI incidence and severity following cardiac surgery: an open-label phase IV randomised pilot study</t>
+    <t>SCR_000025</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>SCR_000025</t>
+    <r>
+      <t xml:space="preserve">Cardiovascular Outcomes of Perioperative Sodium-Glucose Transporter 2 Inhibition in Cardiac Surgery Patients: An Open-Label </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Randomized </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Pilot Study.</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Journal Article; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Randomized Controlled Trial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>; JOUR; Journal article</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Randomized Controlled Trial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>; Journal Article; JOUR; Journal article</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Journal Article; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Randomized Controlled Trial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>; Pragmatic Clinical Trial; JOUR; Journal article</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Journal Article; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Randomized Controlled Trial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>; Research Support, Non-U.S. Gov't; JOUR; Journal article</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SCR_000024</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>SCR_000024 와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve"> 같은 환자군 (Same RCT)</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Journal Article; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Randomized Controlled Trial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>; Clinical Trial, Phase IV; JOUR; Journal article</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The effects of sodium-glucose transporter 2 inhibition on cardiac surgery-associated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>acute kidney injury</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>: An open-label randomized pilot study.</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Evaluation of the effect of empagliflozin on prevention of atrial fibrillation after coronary artery bypass grafting: a double-blind, randomized, placebo-controlled trial.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">JOUR; Journal article; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>RCT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Conference proceeding</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Empagliflozin limits </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>AKI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> incidence and severity following cardiac surgery: an open-label phase IV randomised pilot study</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SGLT2 inhibition reduces cardiac surgery-associated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>acute kidney injury</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>: an open-label randomized study</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SCR_000024 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve"> 같은 환자군 (Same RCT), </t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Evaluation of the effect of empagliflozin on prevention of atrial fibrillation after heart valve surgery: a double-blind, randomized, placebo-controlled trial.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Indian journal of thoracic and cardiovascular surgery</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Journal Article, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>RCT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>Dapagliflozin and</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Acute Kidney Injury</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Following Cardiac Surgery: A Randomized Clinical Trial.</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SCR_000080</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Available</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SCR_000083</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Full-text PDF</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Differential Effects of GLP-1 Receptor Agonist and SGLT2 Inhibitor Add-on Therapy on Outcomes Following Cardiac Surgery: A Propensity Score-Matched Analysis.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impact of preoperative and postoperative modern guideline-directed medical therapy on survival following coronary artery bypass grafting.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SGLT2 Inhibition as a Perioperative Cardiorenal Stabilizer in Cardiac Surgery: Integrated Clinical Cohort and Pleiotropic Network-Based Pharmacological Analysis.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Preoperative Exposure to Sodium-Glucose Cotransporter-2 Inhibitors and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Acute Kidney Injury </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>After Cardiac Surgery: A Retrospective Single-Centre Cohort Study With Overlap Weighting Propensity Score Analysis.</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Perioperative dapagliflozin in diabetic patients undergoing cardiac surgery: the DAPA-CS trial.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Preoperative SGLT2i therapy and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>acute kidney injury</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> in patients undergoing emergency and urgent coronary artery bypass grafting - A causal inference framework.</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Impact of Sodium-Glucose Cotransporter 2 Inhibitors on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Acute Kidney Injury </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Post Off-Pump Coronary Artery Bypass Grafting: A Retrospective Cohort Study and Meta-Analysis.</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Metabolic acidosis in patients with diabetes 2 undergoing cardiac surgery: The impact of SGLT2 inhibitor use: a retrospective cohort study.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SCR_000167</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Postcardiac Surgery Euglycemic Diabetic Ketoacidosis in Patients on Sodium-Glucose Cotransporter 2 Inhibitors.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sodium-glucose cotransport-2 inhibitor induced ketoacidosis following coronary artery bypass surgery: implications for management.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Effects of Sodium-Glucose Transporter 2 Inhibitors (SGLT2-I) in Patients With Ischemic Heart Disease (IHD) Treated by Coronary Artery Bypass Grafting via MiECC: Inflammatory Burden, and Clinical Outcomes at 5 Years of Follow-Up.</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">The abstract describes an open-label randomized pilot trial in adult patients undergoing elective cardiac surgery with cardiopulmonary bypass, comparing perioperative empagliflozin (started 3 days pre-op to 2 days post-op) versus standard care, and reports efficacy (CSA-AKI incidence) and safety outcomes. </t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Conference proceeding, SCR_000024 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>같은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="돋움"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>환자군</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Same RCT);March 2022 and April 2023, 60 patients</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>SCR_000027</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Preoperative dapagliflozin use and cardiac surgery-associated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>acute kidney injury</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>: A single-center retrospective cohort study.</t>
+    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -1360,7 +1898,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1397,6 +1935,38 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="돋움"/>
+      <family val="2"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1436,13 +2006,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1740,19 +2310,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.73046875" customWidth="1"/>
-    <col min="2" max="2" width="95.73046875" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="95.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.45">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B1" s="5"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1760,7 +2330,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1768,7 +2338,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1776,7 +2346,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1784,7 +2354,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1792,7 +2362,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -1800,7 +2370,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1808,7 +2378,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -1816,7 +2386,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1824,7 +2394,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1832,7 +2402,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1840,7 +2410,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1861,56 +2431,56 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U33"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="230.59765625" customWidth="1"/>
-    <col min="2" max="2" width="55.73046875" customWidth="1"/>
-    <col min="3" max="3" width="250.73046875" customWidth="1"/>
+    <col min="1" max="1" width="230.5703125" customWidth="1"/>
+    <col min="2" max="2" width="55.7109375" customWidth="1"/>
+    <col min="3" max="3" width="250.7109375" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="90.53125" customWidth="1"/>
+    <col min="5" max="5" width="90.5703125" customWidth="1"/>
     <col min="6" max="6" width="43" customWidth="1"/>
-    <col min="7" max="7" width="11.265625" customWidth="1"/>
-    <col min="8" max="8" width="140.73046875" customWidth="1"/>
-    <col min="9" max="9" width="9.9296875" customWidth="1"/>
-    <col min="10" max="10" width="123.59765625" customWidth="1"/>
-    <col min="11" max="11" width="12.59765625" customWidth="1"/>
-    <col min="12" max="12" width="55.73046875" customWidth="1"/>
-    <col min="13" max="13" width="40.33203125" customWidth="1"/>
-    <col min="14" max="14" width="28.46484375" customWidth="1"/>
-    <col min="15" max="15" width="27.73046875" customWidth="1"/>
-    <col min="16" max="16" width="37.73046875" customWidth="1"/>
-    <col min="17" max="17" width="16.73046875" customWidth="1"/>
-    <col min="18" max="18" width="21.73046875" customWidth="1"/>
-    <col min="19" max="20" width="250.73046875" customWidth="1"/>
-    <col min="21" max="21" width="25.796875" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" customWidth="1"/>
+    <col min="8" max="8" width="140.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="123.5703125" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" customWidth="1"/>
+    <col min="12" max="12" width="55.7109375" customWidth="1"/>
+    <col min="13" max="13" width="40.28515625" customWidth="1"/>
+    <col min="14" max="14" width="28.42578125" customWidth="1"/>
+    <col min="15" max="15" width="27.7109375" customWidth="1"/>
+    <col min="16" max="16" width="37.7109375" customWidth="1"/>
+    <col min="17" max="17" width="16.7109375" customWidth="1"/>
+    <col min="18" max="18" width="21.7109375" customWidth="1"/>
+    <col min="19" max="20" width="250.7109375" customWidth="1"/>
+    <col min="21" max="21" width="25.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="18" x14ac:dyDescent="0.45">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:21" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>26</v>
       </c>
@@ -1975,7 +2545,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>47</v>
       </c>
@@ -2040,7 +2610,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>67</v>
       </c>
@@ -2105,7 +2675,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>80</v>
       </c>
@@ -2170,7 +2740,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>92</v>
       </c>
@@ -2235,7 +2805,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>105</v>
       </c>
@@ -2300,7 +2870,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>117</v>
       </c>
@@ -2357,7 +2927,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>130</v>
       </c>
@@ -2414,7 +2984,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>141</v>
       </c>
@@ -2475,7 +3045,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>156</v>
       </c>
@@ -2536,7 +3106,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>168</v>
       </c>
@@ -2599,7 +3169,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>180</v>
       </c>
@@ -2660,7 +3230,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>192</v>
       </c>
@@ -2721,7 +3291,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>203</v>
       </c>
@@ -2782,7 +3352,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>216</v>
       </c>
@@ -2843,7 +3413,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>227</v>
       </c>
@@ -2908,7 +3478,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="57" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>238</v>
       </c>
@@ -2973,7 +3543,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>249</v>
       </c>
@@ -3038,7 +3608,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>260</v>
       </c>
@@ -3103,7 +3673,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>273</v>
       </c>
@@ -3168,7 +3738,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>284</v>
       </c>
@@ -3233,7 +3803,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>294</v>
       </c>
@@ -3298,7 +3868,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>305</v>
       </c>
@@ -3363,7 +3933,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>316</v>
       </c>
@@ -3428,7 +3998,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="27" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>328</v>
       </c>
@@ -3489,7 +4059,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="28" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>339</v>
       </c>
@@ -3554,7 +4124,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>349</v>
       </c>
@@ -3615,7 +4185,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>360</v>
       </c>
@@ -3676,7 +4246,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>372</v>
       </c>
@@ -3737,7 +4307,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>382</v>
       </c>
@@ -3798,7 +4368,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="57" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>394</v>
       </c>
@@ -3877,60 +4447,60 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X43"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.19921875" customWidth="1"/>
-    <col min="2" max="2" width="55.73046875" customWidth="1"/>
-    <col min="3" max="3" width="36.53125" customWidth="1"/>
+    <col min="1" max="1" width="24.140625" customWidth="1"/>
+    <col min="2" max="2" width="55.7109375" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="34.796875" customWidth="1"/>
-    <col min="6" max="6" width="21.86328125" customWidth="1"/>
-    <col min="7" max="7" width="11.265625" customWidth="1"/>
-    <col min="8" max="8" width="27.3984375" customWidth="1"/>
-    <col min="9" max="9" width="9.9296875" customWidth="1"/>
-    <col min="10" max="10" width="67.59765625" customWidth="1"/>
-    <col min="11" max="11" width="12.59765625" customWidth="1"/>
-    <col min="12" max="12" width="40.19921875" customWidth="1"/>
-    <col min="13" max="13" width="23.19921875" customWidth="1"/>
-    <col min="14" max="14" width="24.1328125" customWidth="1"/>
-    <col min="15" max="15" width="16.73046875" customWidth="1"/>
-    <col min="16" max="16" width="21.73046875" customWidth="1"/>
-    <col min="17" max="18" width="250.73046875" customWidth="1"/>
-    <col min="19" max="19" width="15.73046875" customWidth="1"/>
-    <col min="20" max="20" width="21.73046875" customWidth="1"/>
-    <col min="21" max="21" width="29.73046875" customWidth="1"/>
-    <col min="22" max="22" width="12.73046875" customWidth="1"/>
-    <col min="23" max="23" width="18.73046875" customWidth="1"/>
+    <col min="5" max="5" width="34.85546875" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" customWidth="1"/>
+    <col min="8" max="8" width="27.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="67.5703125" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" customWidth="1"/>
+    <col min="12" max="12" width="40.140625" customWidth="1"/>
+    <col min="13" max="13" width="23.140625" customWidth="1"/>
+    <col min="14" max="14" width="24.140625" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="21.7109375" customWidth="1"/>
+    <col min="17" max="18" width="250.7109375" customWidth="1"/>
+    <col min="19" max="19" width="15.7109375" customWidth="1"/>
+    <col min="20" max="20" width="21.7109375" customWidth="1"/>
+    <col min="21" max="21" width="29.7109375" customWidth="1"/>
+    <col min="22" max="22" width="12.7109375" customWidth="1"/>
+    <col min="23" max="23" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="18" x14ac:dyDescent="0.45">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>26</v>
       </c>
@@ -4001,12 +4571,12 @@
         <v>411</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:24" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>48</v>
+      <c r="B4" s="3" t="s">
+        <v>441</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>49</v>
@@ -4023,8 +4593,8 @@
       <c r="G4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>54</v>
+      <c r="H4" s="3" t="s">
+        <v>442</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>55</v>
@@ -4059,13 +4629,17 @@
       <c r="S4" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T4" s="2"/>
+      <c r="T4" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
+      <c r="V4" s="3" t="s">
+        <v>447</v>
+      </c>
       <c r="W4" s="2"/>
       <c r="X4" s="2"/>
     </row>
-    <row r="5" spans="1:24" ht="57" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:24" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>67</v>
       </c>
@@ -4087,8 +4661,8 @@
       <c r="G5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>74</v>
+      <c r="H5" s="3" t="s">
+        <v>443</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>55</v>
@@ -4123,13 +4697,15 @@
       <c r="S5" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T5" s="2"/>
+      <c r="T5" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
       <c r="X5" s="2"/>
     </row>
-    <row r="6" spans="1:24" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:24" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>80</v>
       </c>
@@ -4151,8 +4727,8 @@
       <c r="G6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>86</v>
+      <c r="H6" s="3" t="s">
+        <v>444</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>55</v>
@@ -4187,18 +4763,20 @@
       <c r="S6" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T6" s="2"/>
+      <c r="T6" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
       <c r="X6" s="2"/>
     </row>
-    <row r="7" spans="1:24" ht="57" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:24" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>93</v>
+      <c r="B7" s="3" t="s">
+        <v>450</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>94</v>
@@ -4215,8 +4793,8 @@
       <c r="G7" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>99</v>
+      <c r="H7" s="3" t="s">
+        <v>445</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>55</v>
@@ -4251,18 +4829,20 @@
       <c r="S7" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T7" s="2"/>
+      <c r="T7" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
     </row>
-    <row r="8" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A8" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>106</v>
+    <row r="8" spans="1:24" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>449</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>107</v>
@@ -4279,8 +4859,8 @@
       <c r="G8" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>111</v>
+      <c r="H8" s="3" t="s">
+        <v>448</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>55</v>
@@ -4288,8 +4868,8 @@
       <c r="J8" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>57</v>
+      <c r="K8" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>113</v>
@@ -4303,8 +4883,8 @@
       <c r="O8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="P8" s="2" t="s">
-        <v>63</v>
+      <c r="P8" s="3" t="s">
+        <v>462</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>114</v>
@@ -4315,18 +4895,20 @@
       <c r="S8" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T8" s="2"/>
+      <c r="T8" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
       <c r="X8" s="2"/>
     </row>
-    <row r="9" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="A9" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="B9" s="5" t="s">
+    <row r="9" spans="1:24" ht="135" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>440</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>452</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>119</v>
@@ -4341,15 +4923,15 @@
         <v>121</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2" t="s">
-        <v>122</v>
+      <c r="H9" s="3" t="s">
+        <v>451</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>124</v>
+      <c r="K9" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>125</v>
@@ -4367,24 +4949,30 @@
       <c r="Q9" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="R9" s="2" t="s">
-        <v>128</v>
+      <c r="R9" s="3" t="s">
+        <v>475</v>
       </c>
       <c r="S9" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
+      <c r="T9" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="V9" s="3" t="s">
+        <v>476</v>
+      </c>
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
     </row>
-    <row r="10" spans="1:24" ht="57" x14ac:dyDescent="0.45">
-      <c r="A10" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>131</v>
+    <row r="10" spans="1:24" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>453</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>132</v>
@@ -4406,8 +4994,8 @@
       <c r="J10" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>124</v>
+      <c r="K10" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>137</v>
@@ -4419,8 +5007,8 @@
       <c r="O10" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="P10" s="2" t="s">
-        <v>126</v>
+      <c r="P10" s="3" t="s">
+        <v>462</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>138</v>
@@ -4431,13 +5019,19 @@
       <c r="S10" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
+      <c r="T10" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="V10" s="3" t="s">
+        <v>454</v>
+      </c>
       <c r="W10" s="2"/>
       <c r="X10" s="2"/>
     </row>
-    <row r="11" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>141</v>
       </c>
@@ -4501,7 +5095,7 @@
       <c r="W11" s="2"/>
       <c r="X11" s="2"/>
     </row>
-    <row r="12" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>156</v>
       </c>
@@ -4565,7 +5159,7 @@
       <c r="W12" s="2"/>
       <c r="X12" s="2"/>
     </row>
-    <row r="13" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>168</v>
       </c>
@@ -4594,8 +5188,8 @@
       <c r="J13" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="K13" s="2" t="s">
-        <v>57</v>
+      <c r="K13" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>176</v>
@@ -4609,8 +5203,8 @@
       <c r="O13" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="P13" s="2" t="s">
-        <v>63</v>
+      <c r="P13" s="3" t="s">
+        <v>462</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>177</v>
@@ -4621,18 +5215,20 @@
       <c r="S13" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T13" s="2"/>
+      <c r="T13" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
       <c r="X13" s="2"/>
     </row>
-    <row r="14" spans="1:24" ht="57" x14ac:dyDescent="0.45">
-      <c r="A14" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>181</v>
+    <row r="14" spans="1:24" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>455</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>182</v>
@@ -4640,8 +5236,8 @@
       <c r="D14" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>183</v>
+      <c r="E14" s="3" t="s">
+        <v>456</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>184</v>
@@ -4649,8 +5245,8 @@
       <c r="G14" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>186</v>
+      <c r="H14" s="3" t="s">
+        <v>457</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>55</v>
@@ -4658,8 +5254,8 @@
       <c r="J14" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>124</v>
+      <c r="K14" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>188</v>
@@ -4671,8 +5267,8 @@
       <c r="O14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="P14" s="2" t="s">
-        <v>126</v>
+      <c r="P14" s="3" t="s">
+        <v>462</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>189</v>
@@ -4683,18 +5279,20 @@
       <c r="S14" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T14" s="2"/>
+      <c r="T14" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
       <c r="X14" s="2"/>
     </row>
-    <row r="15" spans="1:24" ht="114" x14ac:dyDescent="0.45">
-      <c r="A15" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>193</v>
+    <row r="15" spans="1:24" ht="120" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>458</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>194</v>
@@ -4711,8 +5309,8 @@
       <c r="G15" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>186</v>
+      <c r="H15" s="3" t="s">
+        <v>457</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>55</v>
@@ -4720,8 +5318,8 @@
       <c r="J15" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>124</v>
+      <c r="K15" s="3" t="s">
+        <v>460</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>199</v>
@@ -4733,8 +5331,8 @@
       <c r="O15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="P15" s="2" t="s">
-        <v>126</v>
+      <c r="P15" s="3" t="s">
+        <v>462</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>200</v>
@@ -4745,18 +5343,20 @@
       <c r="S15" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T15" s="2"/>
+      <c r="T15" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
       <c r="X15" s="2"/>
     </row>
-    <row r="16" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>204</v>
+      <c r="B16" s="3" t="s">
+        <v>463</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>205</v>
@@ -4807,18 +5407,20 @@
       <c r="S16" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T16" s="2"/>
+      <c r="T16" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="W16" s="2"/>
       <c r="X16" s="2"/>
     </row>
-    <row r="17" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>216</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>217</v>
+        <v>464</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>218</v>
@@ -4869,18 +5471,22 @@
       <c r="S17" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
+      <c r="T17" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>427</v>
+      </c>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
       <c r="X17" s="2"/>
     </row>
-    <row r="18" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>228</v>
+      <c r="B18" s="3" t="s">
+        <v>465</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>229</v>
@@ -4933,18 +5539,20 @@
       <c r="S18" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T18" s="2"/>
+      <c r="T18" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
     </row>
-    <row r="19" spans="1:24" ht="57" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:24" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>239</v>
+      <c r="B19" s="3" t="s">
+        <v>466</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>240</v>
@@ -4997,18 +5605,20 @@
       <c r="S19" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T19" s="2"/>
+      <c r="T19" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="W19" s="2"/>
       <c r="X19" s="2"/>
     </row>
-    <row r="20" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>250</v>
+      <c r="B20" s="3" t="s">
+        <v>467</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>251</v>
@@ -5061,13 +5671,15 @@
       <c r="S20" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T20" s="2"/>
+      <c r="T20" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2"/>
       <c r="X20" s="2"/>
     </row>
-    <row r="21" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>260</v>
       </c>
@@ -5135,7 +5747,7 @@
       <c r="W21" s="2"/>
       <c r="X21" s="2"/>
     </row>
-    <row r="22" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>273</v>
       </c>
@@ -5201,7 +5813,7 @@
       <c r="W22" s="2"/>
       <c r="X22" s="2"/>
     </row>
-    <row r="23" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>284</v>
       </c>
@@ -5267,12 +5879,12 @@
       <c r="W23" s="2"/>
       <c r="X23" s="2"/>
     </row>
-    <row r="24" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>295</v>
+      <c r="B24" s="3" t="s">
+        <v>469</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>296</v>
@@ -5325,17 +5937,19 @@
       <c r="S24" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T24" s="2"/>
+      <c r="T24" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
       <c r="W24" s="2"/>
     </row>
-    <row r="25" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>306</v>
+      <c r="B25" s="3" t="s">
+        <v>468</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>307</v>
@@ -5388,12 +6002,14 @@
       <c r="S25" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T25" s="2"/>
+      <c r="T25" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
       <c r="W25" s="2"/>
     </row>
-    <row r="26" spans="1:24" ht="57" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:24" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>316</v>
       </c>
@@ -5451,12 +6067,14 @@
       <c r="S26" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T26" s="2"/>
+      <c r="T26" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
       <c r="W26" s="2"/>
     </row>
-    <row r="27" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>328</v>
       </c>
@@ -5512,12 +6130,14 @@
       <c r="S27" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T27" s="2"/>
+      <c r="T27" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
     </row>
-    <row r="28" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:24" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>339</v>
       </c>
@@ -5575,17 +6195,19 @@
       <c r="S28" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T28" s="2"/>
+      <c r="T28" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
     </row>
-    <row r="29" spans="1:24" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>350</v>
+      <c r="B29" s="3" t="s">
+        <v>478</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>351</v>
@@ -5636,17 +6258,19 @@
       <c r="S29" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T29" s="2"/>
+      <c r="T29" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
     </row>
-    <row r="30" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>361</v>
+        <v>471</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>470</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>362</v>
@@ -5697,17 +6321,21 @@
       <c r="S30" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
+      <c r="T30" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="U30" s="2" t="s">
+        <v>425</v>
+      </c>
       <c r="V30" s="2"/>
       <c r="W30" s="2"/>
     </row>
-    <row r="31" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>373</v>
+      <c r="B31" s="3" t="s">
+        <v>472</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>374</v>
@@ -5758,17 +6386,21 @@
       <c r="S31" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T31" s="2"/>
-      <c r="U31" s="2"/>
+      <c r="T31" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="U31" s="2" t="s">
+        <v>425</v>
+      </c>
       <c r="V31" s="2"/>
       <c r="W31" s="2"/>
     </row>
-    <row r="32" spans="1:24" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:24" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>383</v>
+      <c r="B32" s="3" t="s">
+        <v>473</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>384</v>
@@ -5820,18 +6452,20 @@
         <v>412</v>
       </c>
       <c r="T32" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U32" s="2"/>
+        <v>150</v>
+      </c>
+      <c r="U32" s="2" t="s">
+        <v>425</v>
+      </c>
       <c r="V32" s="2"/>
       <c r="W32" s="2"/>
     </row>
-    <row r="33" spans="1:24" ht="57" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:24" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>395</v>
+      <c r="B33" s="3" t="s">
+        <v>474</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>396</v>
@@ -5884,47 +6518,49 @@
       <c r="S33" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="T33" s="2"/>
+      <c r="T33" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
       <c r="W33" s="2"/>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X34" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X35" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X36" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X37" s="2"/>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X38" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X39" s="2"/>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X40" s="2"/>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X41" s="2"/>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X42" s="2"/>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
       <c r="X43" s="2" t="s">
         <v>61</v>
       </c>
@@ -5961,9 +6597,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>413</v>
       </c>
@@ -5980,7 +6616,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -5997,7 +6633,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>150</v>
       </c>
@@ -6014,7 +6650,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>211</v>
       </c>
@@ -6028,7 +6664,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
         <v>424</v>
       </c>
@@ -6036,7 +6672,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>426</v>
       </c>
@@ -6044,7 +6680,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>163</v>
       </c>
@@ -6052,7 +6688,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>151</v>
       </c>
@@ -6060,7 +6696,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>428</v>
       </c>
@@ -6068,7 +6704,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>268</v>
       </c>
@@ -6076,7 +6712,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>430</v>
       </c>
@@ -6084,7 +6720,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>432</v>
       </c>
@@ -6092,7 +6728,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>434</v>
       </c>
@@ -6100,7 +6736,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
         <v>436</v>
       </c>
@@ -6108,7 +6744,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
         <v>438</v>
       </c>

</xml_diff>